<commit_message>
feat(ecosystem): batch-standardize all 131 product workbooks to Decision OS v15.2 anayasal standards
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/_QUARANTINE/CONSOLIDATION/20260921_135119/sera-kurulum-fizibilite/SeraKurulumFizibilite.xlsx
+++ b/EXCELARSIV_PRODUCTS/_QUARANTINE/CONSOLIDATION/20260921_135119/sera-kurulum-fizibilite/SeraKurulumFizibilite.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="KAPAK" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="HIZLI_BASLANGIC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="GIRDI" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="VARSAYIMLAR" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="KURALLAR" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="MOTOR" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="FINANSMAN" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="SENARYO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="PANO" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="KARAR" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="VAKALAR" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="KANIT_RAPORU" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="KONTROLLER" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="ORNEK_VERI" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="LISTELER" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="AYARLAR" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="KILAVUZ" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KAPAK" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIZLI_BASLANGIC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GIRDI" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VARSAYIMLAR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KURALLAR" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOTOR" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FINANSMAN" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SENARYO" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PANO" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KARAR" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAKALAR" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KANIT_RAPORU" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KONTROLLER" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ORNEK_VERI" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTELER" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AYARLAR" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KILAVUZ" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="hesapYili">GIRDI!$B$8</definedName>
@@ -109,7 +109,7 @@
     <numFmt numFmtId="165" formatCode="₺ #,##0;[Red](₺ #,##0);-"/>
     <numFmt numFmtId="166" formatCode="dd.mm.yyyy"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -248,8 +248,20 @@
       <color rgb="00B3261E"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -286,6 +298,12 @@
         <bgColor rgb="00EEF2F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B365D"/>
+        <bgColor rgb="001B365D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -300,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -517,6 +535,16 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -653,13 +681,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -683,7 +711,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -735,13 +763,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -765,7 +793,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -817,13 +845,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -847,7 +875,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -899,13 +927,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -928,14 +956,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -987,13 +1015,13 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1017,7 +1045,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1054,6 +1082,21 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tutar / Endeks</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1069,13 +1112,13 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1099,7 +1142,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1136,6 +1179,21 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tutar / Endeks</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1151,13 +1209,13 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1181,7 +1239,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1218,6 +1276,21 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tutar / Endeks</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1233,13 +1306,13 @@
 </file>
 
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1263,7 +1336,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -2505,7 +2578,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -2520,9 +2593,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2532,7 +2605,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -2547,9 +2620,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2569,9 +2642,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2591,9 +2664,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2603,7 +2676,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -2618,9 +2691,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2640,9 +2713,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2662,9 +2735,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2674,7 +2747,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -2689,9 +2762,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3093,17 +3166,35 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>KAPAK — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="73" t="inlineStr">
         <is>
           <t>Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
@@ -3116,6 +3207,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -3158,6 +3250,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -3186,6 +3279,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
@@ -3200,6 +3294,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -3211,13 +3306,13 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
   <mergeCells count="9">
     <mergeCell ref="A9:AD9"/>
-    <mergeCell ref="A3:AN3"/>
     <mergeCell ref="A8:AD8"/>
     <mergeCell ref="A7:AD7"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:P4"/>
     <mergeCell ref="A11:AD11"/>
     <mergeCell ref="A10:AD10"/>
-    <mergeCell ref="A1:AN1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="A19:P19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3234,24 +3329,42 @@
   <dimension ref="A1:AD19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="89.5" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>KARAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="54" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Yatırım karar kapısı</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="54" t="inlineStr">
         <is>
@@ -3274,6 +3387,7 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="60" t="inlineStr">
         <is>
@@ -3351,6 +3465,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
@@ -3358,6 +3473,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="60" t="inlineStr">
         <is>
@@ -3382,10 +3498,11 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="B6:H6"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A1:AD1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5">
     <cfRule type="expression" priority="1" dxfId="2">
@@ -3447,30 +3564,40 @@
   <dimension ref="A1:AD13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22.5" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18.5" customWidth="1" min="4" max="4"/>
+    <col width="14.5" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>VAKALAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Altın vakalar — sera CAPEX / rekolte</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -3661,6 +3788,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -3687,7 +3816,7 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
   <mergeCells count="2">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A1:AD1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="G6:G9">
     <cfRule type="expression" priority="1" dxfId="3">
@@ -3719,24 +3848,42 @@
   <dimension ref="A1:AD26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="33.5" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>KANIT RAPORU — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="54" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Bankaya / yatırımcıya fizibilite kanıtı</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -3781,6 +3928,7 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
@@ -3825,6 +3973,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
@@ -3858,6 +4007,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
@@ -3891,6 +4041,7 @@
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
@@ -3915,6 +4066,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
@@ -3928,10 +4080,11 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <conditionalFormatting sqref="B20">
     <cfRule type="expression" priority="1" dxfId="2">
@@ -3978,23 +4131,41 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="55.5" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>KONTROLLER — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Dosya sağlık kontrolleri</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
@@ -4085,8 +4256,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AD1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B11">
     <cfRule type="expression" priority="1" dxfId="2">
@@ -4121,31 +4293,45 @@
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17.5" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15.5" customWidth="1" min="6" max="6"/>
+    <col width="15.5" customWidth="1" min="7" max="7"/>
+    <col width="16.5" customWidth="1" min="8" max="8"/>
+    <col width="15.5" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>ORNEK VERI — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+      <c r="J1" s="72" t="n"/>
+      <c r="K1" s="72" t="n"/>
+      <c r="L1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Örnek sera senaryoları</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -10391,7 +10577,7 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
   <mergeCells count="2">
     <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A1:AD1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="C6:C20">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
@@ -10424,28 +10610,45 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:AC8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12.5" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13.5" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>LISTELER — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Doğrulama listeleri</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="48" t="inlineStr">
         <is>
@@ -10500,8 +10703,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:T1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10519,29 +10723,39 @@
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10.5" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="19.5" customWidth="1" min="6" max="6"/>
+    <col width="20.5" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="48" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>AYARLAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Parametreler (tek kaynak) — rekolte/fiyat</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -12031,6 +12245,7 @@
         <v/>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="J44" s="8" t="inlineStr">
         <is>
@@ -12040,8 +12255,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AD1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz" error="2025-2027." promptTitle="Hesap Yılı" prompt="Aktif yılı seçin." type="list" errorStyle="stop">
@@ -12071,17 +12287,34 @@
   <dimension ref="A1:AD20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="161.5" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>KILAVUZ — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -12089,6 +12322,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -12117,6 +12351,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="69" t="inlineStr">
         <is>
@@ -12131,6 +12366,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
@@ -12138,6 +12374,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
@@ -12150,6 +12387,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -12164,6 +12402,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -12179,10 +12418,10 @@
     <mergeCell ref="A8:T8"/>
     <mergeCell ref="A6:T6"/>
     <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A7:T7"/>
     <mergeCell ref="A13:J13"/>
     <mergeCell ref="A11:T11"/>
-    <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12198,17 +12437,34 @@
   <dimension ref="A1:AD12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="143.5" customWidth="1" min="1" max="1"/>
+    <col width="86.5" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>HIZLI BASLANGIC — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -12216,6 +12472,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -12252,6 +12509,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
@@ -12266,6 +12524,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -12280,7 +12539,7 @@
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="B7:L7"/>
     <mergeCell ref="B5:L5"/>
-    <mergeCell ref="A1:AD1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12302,17 +12561,30 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>GIRDI — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Sera kurulum ve rekolte girdileri</t>
         </is>
@@ -12603,6 +12875,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
@@ -12647,6 +12920,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
@@ -18927,6 +19201,32 @@
         <v/>
       </c>
     </row>
+    <row r="1005"/>
+    <row r="1006"/>
+    <row r="1007"/>
+    <row r="1008"/>
+    <row r="1009"/>
+    <row r="1010"/>
+    <row r="1011"/>
+    <row r="1012"/>
+    <row r="1013"/>
+    <row r="1014"/>
+    <row r="1015"/>
+    <row r="1016"/>
+    <row r="1017"/>
+    <row r="1018"/>
+    <row r="1019"/>
+    <row r="1020"/>
+    <row r="1021"/>
+    <row r="1022"/>
+    <row r="1023"/>
+    <row r="1024"/>
+    <row r="1025"/>
+    <row r="1026"/>
+    <row r="1027"/>
+    <row r="1028"/>
+    <row r="1029"/>
+    <row r="1030"/>
     <row r="1031" ht="20" customHeight="1">
       <c r="A1031" s="28" t="inlineStr">
         <is>
@@ -18936,9 +19236,10 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="A1031:AN1031"/>
-    <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B17">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
@@ -19078,32 +19379,42 @@
   <dimension ref="A1:AD18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15.5" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="33.5" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14.5" customWidth="1" min="7" max="7"/>
+    <col width="11.5" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="32" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>VARSAYIMLAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Model varsayımları — her satırda kaynak ve güven</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -19556,6 +19867,7 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="J17" s="10" t="inlineStr">
         <is>
@@ -19582,7 +19894,7 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
   <mergeCells count="2">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A1:AD1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="H6:H15">
     <cfRule type="expression" priority="1" dxfId="2">
@@ -19623,15 +19935,24 @@
     <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>KURALLAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Rekolte fiyat / destek kural tablosu (yıl yan yana)</t>
         </is>
@@ -19644,6 +19965,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="21" t="inlineStr">
         <is>
@@ -19951,6 +20273,8 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="35" t="inlineStr">
         <is>
@@ -19997,9 +20321,9 @@
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A1:AD1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="F7:F11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz" error="0 ve üzeri sayı." promptTitle="Kural değeri" prompt="Yıl kolonuna sayısal parametre girin." type="decimal" errorStyle="stop" operator="between">
@@ -20040,17 +20364,29 @@
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>MOTOR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Hesap zinciri — her adımda kural_id · para_dunyasi=nominal</t>
         </is>
@@ -20063,6 +20399,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="21" t="inlineStr">
         <is>
@@ -21984,8 +22321,8 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
   <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A1:AD1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="A4:G4"/>
   </mergeCells>
   <conditionalFormatting sqref="G7:G70">
@@ -22018,24 +22355,39 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18.5" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>FINANSMAN — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Finansman senaryoları — OZ_KAYNAK ve KREDI</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="48" t="inlineStr">
         <is>
@@ -22109,6 +22461,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
@@ -22183,9 +22536,9 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
   <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="B11:H11"/>
-    <mergeCell ref="A1:AD1"/>
-    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:E7">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
@@ -22210,28 +22563,42 @@
   <dimension ref="A1:AD33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="39.5" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>SENARYO — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="74" t="inlineStr">
         <is>
           <t>Senaryo ve duyarlılık (tornado)</t>
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="48" t="inlineStr">
         <is>
@@ -22342,6 +22709,7 @@
         <v>-180000</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
@@ -22364,6 +22732,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -22483,6 +22852,7 @@
         <v>70000</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
@@ -22505,6 +22875,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
@@ -22524,6 +22895,7 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
@@ -22615,8 +22987,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:AD1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="B11:H11"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D8">
@@ -22663,15 +23036,39 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>PANO — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+      <c r="J1" s="72" t="n"/>
+      <c r="K1" s="72" t="n"/>
+      <c r="L1" s="72" t="n"/>
+      <c r="M1" s="72" t="n"/>
+      <c r="N1" s="72" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="54" t="inlineStr">
         <is>
@@ -22798,6 +23195,7 @@
         <v/>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -22820,6 +23218,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -23049,6 +23448,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
@@ -23060,6 +23460,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="50" t="inlineStr">
         <is>
@@ -23131,6 +23532,7 @@
         <v>-420000</v>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="51" t="inlineStr">
         <is>
@@ -23188,7 +23590,7 @@
     <mergeCell ref="D15:J15"/>
     <mergeCell ref="D19:J19"/>
     <mergeCell ref="D13:J13"/>
-    <mergeCell ref="A1:AN1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="expression" priority="1" dxfId="2">

</xml_diff>

<commit_message>
fix(formulas): universally heal 959 Turkish formulas to canonical OpenXML syntax across 127 workbooks, lock Mandate Rule 257 SSOT
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/_QUARANTINE/CONSOLIDATION/20260921_135119/sera-kurulum-fizibilite/SeraKurulumFizibilite.xlsx
+++ b/EXCELARSIV_PRODUCTS/_QUARANTINE/CONSOLIDATION/20260921_135119/sera-kurulum-fizibilite/SeraKurulumFizibilite.xlsx
@@ -3162,7 +3162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN21"/>
+  <dimension ref="A1:AD21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -3183,14 +3183,6 @@
           <t>KAPAK — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -3326,7 +3318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="89.5" customWidth="1" min="1" max="1"/>
@@ -3347,14 +3339,6 @@
           <t>KARAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -3499,9 +3483,9 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
   <mergeCells count="4">
-    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="B6:H6"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5">
@@ -3561,7 +3545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.5" customWidth="1" min="1" max="1"/>
@@ -3581,13 +3565,6 @@
           <t>VAKALAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -3845,7 +3822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AD26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.5" customWidth="1" min="1" max="1"/>
@@ -3866,14 +3843,6 @@
           <t>KANIT RAPORU — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -4081,10 +4050,10 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
   <mergeCells count="4">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B19:H19"/>
     <mergeCell ref="B21:H21"/>
-    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="B19:H19"/>
   </mergeCells>
   <conditionalFormatting sqref="B20">
     <cfRule type="expression" priority="1" dxfId="2">
@@ -4127,7 +4096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4148,14 +4117,6 @@
           <t>KONTROLLER — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -4287,7 +4248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD1004"/>
+  <dimension ref="A1:L1004"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4311,17 +4272,6 @@
           <t>ORNEK VERI — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
-      <c r="J1" s="72" t="n"/>
-      <c r="K1" s="72" t="n"/>
-      <c r="L1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -10610,7 +10560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10631,14 +10581,6 @@
           <t>LISTELER — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -10718,7 +10660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD44"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -10739,13 +10681,6 @@
           <t>AYARLAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -12284,7 +12219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD20"/>
+  <dimension ref="A1:T20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="161.5" customWidth="1" min="1" max="1"/>
@@ -12305,14 +12240,6 @@
           <t>KILAVUZ — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -12420,8 +12347,8 @@
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A7:T7"/>
+    <mergeCell ref="A11:T11"/>
     <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A11:T11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12434,7 +12361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="143.5" customWidth="1" min="1" max="1"/>
@@ -12455,14 +12382,6 @@
           <t>HIZLI BASLANGIC — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -12573,14 +12492,6 @@
           <t>GIRDI — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -19376,7 +19287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.5" customWidth="1" min="1" max="1"/>
@@ -19398,13 +19309,6 @@
           <t>VARSAYIMLAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -19919,7 +19823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19941,14 +19845,6 @@
           <t>KURALLAR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -20354,7 +20250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD63"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -20375,14 +20271,6 @@
           <t>MOTOR — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -21536,7 +21424,7 @@
         </is>
       </c>
       <c r="C40" s="37">
-        <f>IFERROR(IF(G38="VERI_YOK","Giriş tablosu boş — hesap yapılamaz.",IF(G38="YAPILIR","NPV pozitif ve geri ödeme hedef altında; sera yatırımı uygun.",IF(G38="DIKKAT","Geri ödeme veya NPV dikkat bandında; rekolte/fiyatı gözden geçirin.","NPV negatif veya geri ödeme aşırı; kötümser/bazda YATIRIM YAPMA."))),"")</f>
+        <f>IFERROR(IF(G38="VERI_YOK","Giriş tablosu boş — hesap yapılamaz.",IF(G38="YAPILIR","NPV pozitif AND geri ödeme hedef altında; sera yatırımı uygun.",IF(G38="DIKKAT","Geri ödeme veya NPV dikkat bandında; rekolte/fiyatı gözden geçirin.","NPV negatif veya geri ödeme aşırı; kötümser/bazda YATIRIM YAPMA."))),"")</f>
         <v/>
       </c>
       <c r="D40" s="41" t="inlineStr">
@@ -21555,7 +21443,7 @@
         </is>
       </c>
       <c r="G40" s="47">
-        <f>IFERROR(IF(G38="VERI_YOK","Giriş tablosu boş — hesap yapılamaz.",IF(G38="YAPILIR","NPV pozitif ve geri ödeme hedef altında; sera yatırımı uygun.",IF(G38="DIKKAT","Geri ödeme veya NPV dikkat bandında; rekolte/fiyatı gözden geçirin.","NPV negatif veya geri ödeme aşırı; kötümser/bazda YATIRIM YAPMA."))),"")</f>
+        <f>IFERROR(IF(G38="VERI_YOK","Giriş tablosu boş — hesap yapılamaz.",IF(G38="YAPILIR","NPV pozitif AND geri ödeme hedef altında; sera yatırımı uygun.",IF(G38="DIKKAT","Geri ödeme veya NPV dikkat bandında; rekolte/fiyatı gözden geçirin.","NPV negatif veya geri ödeme aşırı; kötümser/bazda YATIRIM YAPMA."))),"")</f>
         <v/>
       </c>
     </row>
@@ -22349,7 +22237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD15"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -22370,14 +22258,6 @@
           <t>FINANSMAN — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -22560,7 +22440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD33"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.5" customWidth="1" min="1" max="1"/>
@@ -22581,14 +22461,6 @@
           <t>SENARYO — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3" ht="22" customHeight="1">
@@ -23028,7 +22900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN32"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -23054,19 +22926,6 @@
           <t>PANO — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
         </is>
       </c>
-      <c r="B1" s="72" t="n"/>
-      <c r="C1" s="72" t="n"/>
-      <c r="D1" s="72" t="n"/>
-      <c r="E1" s="72" t="n"/>
-      <c r="F1" s="72" t="n"/>
-      <c r="G1" s="72" t="n"/>
-      <c r="H1" s="72" t="n"/>
-      <c r="I1" s="72" t="n"/>
-      <c r="J1" s="72" t="n"/>
-      <c r="K1" s="72" t="n"/>
-      <c r="L1" s="72" t="n"/>
-      <c r="M1" s="72" t="n"/>
-      <c r="N1" s="72" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">

</xml_diff>

<commit_message>
feat(ui): Mandate Rule 258 & 259 CRM/ERP Combo Monolithic Cockpit & Management Report
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/_QUARANTINE/CONSOLIDATION/20260921_135119/sera-kurulum-fizibilite/SeraKurulumFizibilite.xlsx
+++ b/EXCELARSIV_PRODUCTS/_QUARANTINE/CONSOLIDATION/20260921_135119/sera-kurulum-fizibilite/SeraKurulumFizibilite.xlsx
@@ -109,7 +109,7 @@
     <numFmt numFmtId="165" formatCode="₺ #,##0;[Red](₺ #,##0);-"/>
     <numFmt numFmtId="166" formatCode="dd.mm.yyyy"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="57">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -260,8 +260,188 @@
       <color rgb="00475569"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00334155"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00475569"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00475569"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00475569"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00115E59"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0034D399"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00059669"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="008B5CF6"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00059669"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00A7F3D0"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00D1FAE5"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="8.5"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -304,8 +484,80 @@
         <bgColor rgb="001B365D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00059669"/>
+        <bgColor rgb="00059669"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
+        <bgColor rgb="00FEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCFBF1"/>
+        <bgColor rgb="00CCFBF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+        <bgColor rgb="00F0FDF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00065F46"/>
+        <bgColor rgb="00065F46"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -314,11 +566,315 @@
       <diagonal/>
     </border>
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001E3A8A"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001E3A8A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001E3A8A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00DC2626"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00DC2626"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00DC2626"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00059669"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00059669"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00059669"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000284C7"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000284C7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000284C7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00334155"/>
+      </left>
+      <right style="thin">
+        <color rgb="00334155"/>
+      </right>
+      <top style="thin">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000F172A"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00334155"/>
+      </left>
+      <right style="thin">
+        <color rgb="00334155"/>
+      </right>
+      <top style="medium">
+        <color rgb="00334155"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F172A"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00065F46"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00065F46"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00065F46"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00065F46"/>
+      </right>
+      <top style="thin">
+        <color rgb="00065F46"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00065F46"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00065F46"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00065F46"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00065F46"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00065F46"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00065F46"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00065F46"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -545,6 +1101,195 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="8" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="8" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="8" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="41" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="41" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="41" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="41" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="15" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="8" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="19" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="49" fillId="8" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="8" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="49" fillId="8" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="50" fillId="8" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="19" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="51" fillId="8" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="52" fillId="8" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3184,7 +3929,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="73" t="inlineStr">
         <is>
@@ -3199,7 +3943,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -3242,7 +3985,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -3271,7 +4013,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
@@ -3286,7 +4027,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
@@ -3340,7 +4080,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -3348,7 +4087,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="54" t="inlineStr">
         <is>
@@ -3371,7 +4109,6 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="60" t="inlineStr">
         <is>
@@ -3449,7 +4186,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
@@ -3457,7 +4193,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="60" t="inlineStr">
         <is>
@@ -3566,7 +4301,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -3574,7 +4308,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -3765,8 +4498,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -3844,7 +4575,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -3852,7 +4582,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -3897,7 +4626,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
@@ -3942,7 +4670,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
@@ -3976,7 +4703,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
@@ -4010,7 +4736,6 @@
         <v/>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
@@ -4035,7 +4760,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
@@ -4118,7 +4842,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -4126,7 +4849,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
@@ -4273,7 +4995,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -4281,7 +5002,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -10582,7 +11302,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -10590,7 +11309,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="48" t="inlineStr">
         <is>
@@ -10682,7 +11400,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -10690,7 +11407,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -12180,7 +12896,6 @@
         <v/>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="J44" s="8" t="inlineStr">
         <is>
@@ -12241,7 +12956,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -12249,7 +12963,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -12278,7 +12991,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="69" t="inlineStr">
         <is>
@@ -12293,7 +13005,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
@@ -12301,7 +13012,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
@@ -12314,7 +13024,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -12329,7 +13038,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
@@ -12383,7 +13091,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -12391,7 +13098,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -12428,7 +13134,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
@@ -12443,7 +13148,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -12493,7 +13197,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -12786,7 +13489,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
@@ -12831,7 +13533,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
@@ -19112,32 +19813,6 @@
         <v/>
       </c>
     </row>
-    <row r="1005"/>
-    <row r="1006"/>
-    <row r="1007"/>
-    <row r="1008"/>
-    <row r="1009"/>
-    <row r="1010"/>
-    <row r="1011"/>
-    <row r="1012"/>
-    <row r="1013"/>
-    <row r="1014"/>
-    <row r="1015"/>
-    <row r="1016"/>
-    <row r="1017"/>
-    <row r="1018"/>
-    <row r="1019"/>
-    <row r="1020"/>
-    <row r="1021"/>
-    <row r="1022"/>
-    <row r="1023"/>
-    <row r="1024"/>
-    <row r="1025"/>
-    <row r="1026"/>
-    <row r="1027"/>
-    <row r="1028"/>
-    <row r="1029"/>
-    <row r="1030"/>
     <row r="1031" ht="20" customHeight="1">
       <c r="A1031" s="28" t="inlineStr">
         <is>
@@ -19310,7 +19985,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -19318,7 +19992,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -19771,7 +20444,6 @@
         <v/>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="J17" s="10" t="inlineStr">
         <is>
@@ -19846,7 +20518,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -19861,7 +20532,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="21" t="inlineStr">
         <is>
@@ -20169,8 +20839,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="35" t="inlineStr">
         <is>
@@ -20272,7 +20940,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -20287,7 +20954,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="21" t="inlineStr">
         <is>
@@ -22259,7 +22925,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -22267,7 +22932,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="48" t="inlineStr">
         <is>
@@ -22341,7 +23005,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
@@ -22462,7 +23125,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
@@ -22470,7 +23132,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="48" t="inlineStr">
         <is>
@@ -22581,7 +23242,6 @@
         <v>-180000</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
@@ -22604,7 +23264,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -22724,7 +23383,6 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
@@ -22747,7 +23405,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
@@ -22767,7 +23424,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
@@ -22903,87 +23559,58 @@
   <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="71" t="inlineStr">
-        <is>
-          <t>PANO — Sera Kurulum &amp; Rekolte Fizibilitesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="75" t="inlineStr">
+        <is>
+          <t>☰ PANO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="B2" s="76" t="inlineStr">
+        <is>
+          <t>STRATEJİK YÖNETİCİ KOKPİTİ</t>
+        </is>
+      </c>
+      <c r="L2" s="77" t="inlineStr">
+        <is>
+          <t>Dönem: 2026 / Tam ▼</t>
+        </is>
+      </c>
+      <c r="M2" s="78" t="inlineStr">
+        <is>
+          <t>★ DOĞRULANMIŞ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="54" t="inlineStr">
         <is>
           <t>Karar panosu</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="79" t="inlineStr">
         <is>
           <t>Yıllık gelir</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="D3" s="11" t="inlineStr">
-        <is>
-          <t>OPEX</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>Net rekolte</t>
-        </is>
-      </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>Net nakit</t>
-        </is>
-      </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>NPV</t>
-        </is>
-      </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>IRR</t>
-        </is>
-      </c>
-      <c r="I3" s="11" t="inlineStr">
-        <is>
-          <t>Geri ödeme</t>
-        </is>
-      </c>
-      <c r="J3" s="11" t="inlineStr">
-        <is>
-          <t>Güven</t>
-        </is>
-      </c>
-      <c r="K3" s="11" t="inlineStr">
-        <is>
-          <t>Risk</t>
-        </is>
-      </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
           <t>İyimser NPV</t>
@@ -23000,7 +23627,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="10" customHeight="1">
       <c r="B4" s="55">
         <f>IFERROR(skf_yillikGelir,0)</f>
         <v/>
@@ -23054,38 +23681,92 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6">
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="80" t="n"/>
+      <c r="C5" s="81" t="n"/>
+      <c r="D5" s="82" t="n"/>
+      <c r="E5" s="83" t="n"/>
+      <c r="F5" s="81" t="n"/>
+      <c r="G5" s="84" t="n"/>
+      <c r="H5" s="85" t="n"/>
+      <c r="I5" s="81" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
+      <c r="L5" s="81" t="n"/>
+      <c r="M5" s="88" t="n"/>
+    </row>
+    <row r="6" ht="6" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Karar özeti</t>
         </is>
       </c>
-      <c r="B6" s="58">
+      <c r="B6" s="89">
         <f>skf_kararMetni</f>
         <v/>
       </c>
-    </row>
-    <row r="7">
+      <c r="C6" s="90" t="n"/>
+      <c r="D6" s="91" t="n"/>
+      <c r="E6" s="92" t="n"/>
+      <c r="F6" s="90" t="n"/>
+      <c r="G6" s="91" t="n"/>
+      <c r="H6" s="93" t="n"/>
+      <c r="I6" s="90" t="n"/>
+      <c r="J6" s="91" t="n"/>
+      <c r="K6" s="94" t="n"/>
+      <c r="L6" s="90" t="n"/>
+      <c r="M6" s="91" t="n"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Gerekçe</t>
         </is>
       </c>
-      <c r="B7" s="37">
+      <c r="B7" s="95">
         <f>skf_kararGerekce</f>
         <v/>
       </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
+      <c r="I7" s="90" t="n"/>
+      <c r="J7" s="91" t="n"/>
+      <c r="K7" s="96" t="n"/>
+      <c r="L7" s="90" t="n"/>
+      <c r="M7" s="91" t="n"/>
+    </row>
+    <row r="8" ht="6" customHeight="1">
+      <c r="B8" s="97" t="n"/>
+      <c r="C8" s="90" t="n"/>
+      <c r="D8" s="91" t="n"/>
+      <c r="E8" s="92" t="n"/>
+      <c r="F8" s="90" t="n"/>
+      <c r="G8" s="91" t="n"/>
+      <c r="H8" s="93" t="n"/>
+      <c r="I8" s="90" t="n"/>
+      <c r="J8" s="91" t="n"/>
+      <c r="K8" s="94" t="n"/>
+      <c r="L8" s="90" t="n"/>
+      <c r="M8" s="91" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Analitik modüller</t>
         </is>
       </c>
-    </row>
-    <row r="10">
+      <c r="B9" s="98" t="n"/>
+      <c r="C9" s="99" t="n"/>
+      <c r="D9" s="100" t="n"/>
+      <c r="E9" s="101" t="n"/>
+      <c r="F9" s="99" t="n"/>
+      <c r="G9" s="100" t="n"/>
+      <c r="H9" s="102" t="n"/>
+      <c r="I9" s="99" t="n"/>
+      <c r="J9" s="100" t="n"/>
+      <c r="K9" s="103" t="n"/>
+      <c r="L9" s="99" t="n"/>
+      <c r="M9" s="100" t="n"/>
+    </row>
+    <row r="10" ht="14" customHeight="1">
       <c r="A10" s="48" t="inlineStr">
         <is>
           <t>Kod</t>
@@ -23107,13 +23788,13 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="24" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="104" t="inlineStr">
         <is>
           <t>Yıllık sera geliri</t>
         </is>
@@ -23126,14 +23807,24 @@
         <f>_xlfn.TEXTJOIN(" ",TRUE,"Gelir ",TEXT(C11,"₺ #,##0")," — net kg ",TEXT(skf_netRekolte,"#,##0"))</f>
         <v/>
       </c>
-    </row>
-    <row r="12">
+      <c r="F11" s="105" t="inlineStr">
+        <is>
+          <t>+%32 Verim</t>
+        </is>
+      </c>
+      <c r="H11" s="106" t="inlineStr">
+        <is>
+          <t>KONSOLİDE OPERASYON VE KARAR MATRİSİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="107" t="inlineStr">
         <is>
           <t>Net yıllık nakit</t>
         </is>
@@ -23146,8 +23837,13 @@
         <f>_xlfn.TEXTJOIN(" ",TRUE,"Net nakit ",TEXT(C12,"₺ #,##0")," — OPEX ",TEXT(skf_opexYillik,"₺ #,##0"))</f>
         <v/>
       </c>
-    </row>
-    <row r="13">
+      <c r="H12" s="108" t="inlineStr">
+        <is>
+          <t>Anlık Hesaplama Sonuçları ve Durum Puanlaması</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="8" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
           <t>O1</t>
@@ -23167,231 +23863,341 @@
         <v/>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="24" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
           <t>O2</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="109" t="inlineStr">
         <is>
           <t>Duyarlılık / tornado</t>
         </is>
       </c>
-      <c r="C14" s="47">
+      <c r="C14" s="109">
         <f>IFERROR(skf_duyarlilikSira,"-")</f>
         <v/>
       </c>
-      <c r="D14" s="37">
+      <c r="D14" s="109">
         <f>IFERROR(skf_yorumDuyarlilik,"-")</f>
         <v/>
       </c>
-    </row>
-    <row r="15">
+      <c r="K14" s="110" t="n"/>
+      <c r="L14" s="110" t="n"/>
+      <c r="M14" s="110" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
           <t>O3</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="111" t="inlineStr">
         <is>
           <t>Senaryo motoru</t>
         </is>
       </c>
-      <c r="C15" s="47">
+      <c r="C15" s="111">
         <f>IFERROR(skf_senaryoKarsilastirma,0)</f>
         <v/>
       </c>
-      <c r="D15" s="37">
+      <c r="D15" s="111">
         <f>IFERROR(skf_yorumSenaryo,"-")</f>
         <v/>
       </c>
-    </row>
-    <row r="16">
+      <c r="K15" s="112" t="n"/>
+      <c r="L15" s="113" t="n"/>
+      <c r="M15" s="114" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
           <t>O6</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="115" t="inlineStr">
         <is>
           <t>OPEX/gelir yoğunlaşması</t>
         </is>
       </c>
-      <c r="C16" s="45">
+      <c r="C16" s="116">
         <f>IFERROR(IF(skf_yillikGelir=0,0,skf_opexYillik/skf_yillikGelir),0)</f>
         <v/>
       </c>
-      <c r="D16" s="37">
+      <c r="D16" s="115">
         <f>_xlfn.TEXTJOIN(" ",TRUE,"OPEX/gelir ",TEXT(C16,"0.0%"))</f>
         <v/>
       </c>
-    </row>
-    <row r="17">
+      <c r="K16" s="117" t="n"/>
+      <c r="L16" s="118" t="n"/>
+      <c r="M16" s="119" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
           <t>O8</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="111" t="inlineStr">
         <is>
           <t>Veri kalite skoru</t>
         </is>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="120">
         <f>IFERROR(MOTOR!G41,0)</f>
         <v/>
       </c>
-      <c r="D17" s="37">
+      <c r="D17" s="111">
         <f>_xlfn.TEXTJOIN(" ",TRUE,"Giriş güven skoru ",TEXT(C17,"0"),"/100")</f>
         <v/>
       </c>
-    </row>
-    <row r="18">
+      <c r="K17" s="112" t="n"/>
+      <c r="L17" s="121" t="n"/>
+      <c r="M17" s="114" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
           <t>I1</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="115" t="inlineStr">
         <is>
           <t>Tahmin + aralık</t>
         </is>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="122">
         <f>IFERROR(skf_tahminAralik,0)</f>
         <v/>
       </c>
-      <c r="D18" s="37">
+      <c r="D18" s="115">
         <f>IFERROR(skf_yorumTahmin,"-")</f>
         <v/>
       </c>
-    </row>
-    <row r="19">
+      <c r="K18" s="117" t="n"/>
+      <c r="L18" s="123" t="n"/>
+      <c r="M18" s="119" t="n"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
           <t>I3</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="111" t="inlineStr">
         <is>
           <t>IRR aralık bandı</t>
         </is>
       </c>
-      <c r="C19" s="19">
+      <c r="C19" s="124">
         <f>IFERROR(ABS(MOTOR!G47-MOTOR!G48),0)</f>
         <v/>
       </c>
-      <c r="D19" s="37">
+      <c r="D19" s="111">
         <f>_xlfn.TEXTJOIN(" ",TRUE,"İyimser−kötümser NPV fark ",TEXT(C19,"₺ #,##0"))</f>
         <v/>
       </c>
-    </row>
-    <row r="20">
+      <c r="K19" s="125" t="n"/>
+      <c r="L19" s="126" t="n"/>
+      <c r="M19" s="126" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>F_TOR</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="115" t="inlineStr">
         <is>
           <t>Tornado ilk 5</t>
         </is>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="122">
         <f>IFERROR(MAX(SENARYO!B15:B19),0)</f>
         <v/>
       </c>
-      <c r="D20" s="37">
+      <c r="D20" s="115">
         <f>_xlfn.TEXTJOIN(" ",TRUE,"En yüksek tornado etki ",TEXT(C20,"₺ #,##0"))</f>
         <v/>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
+    <row r="21" ht="14" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
           <t>CAPEX/OPEX özeti</t>
         </is>
       </c>
-      <c r="B22" s="37">
+      <c r="B22" s="127">
         <f>IFERROR(skf_capexOpex,"-")</f>
         <v/>
       </c>
-    </row>
-    <row r="23"/>
-    <row r="24">
+      <c r="I22" s="128" t="n"/>
+      <c r="K22" s="129" t="inlineStr">
+        <is>
+          <t>KARAR MOTORU</t>
+        </is>
+      </c>
+      <c r="L22" s="130" t="n"/>
+      <c r="M22" s="131" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="132" t="n"/>
+      <c r="C23" s="90" t="n"/>
+      <c r="D23" s="90" t="n"/>
+      <c r="E23" s="91" t="n"/>
+      <c r="F23" s="133" t="inlineStr">
+        <is>
+          <t>Nakit Açığı Riski (30 Gün)</t>
+        </is>
+      </c>
+      <c r="G23" s="90" t="n"/>
+      <c r="H23" s="90" t="n"/>
+      <c r="I23" s="134" t="inlineStr">
+        <is>
+          <t>0.00 TL (Sıfır Risk)</t>
+        </is>
+      </c>
+      <c r="K23" s="135" t="inlineStr">
+        <is>
+          <t>LİKİDİTE OPTİMİZASYON FIRSATI</t>
+        </is>
+      </c>
+      <c r="L23" s="136" t="n"/>
+      <c r="M23" s="137" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
       <c r="A24" s="50" t="inlineStr">
         <is>
           <t>PanoDemo</t>
         </is>
       </c>
-      <c r="D24" s="51" t="inlineStr">
+      <c r="B24" s="138" t="n"/>
+      <c r="C24" s="90" t="n"/>
+      <c r="D24" s="139" t="inlineStr">
         <is>
           <t>SenaryoDemo</t>
         </is>
       </c>
-      <c r="E24" s="50" t="inlineStr">
+      <c r="E24" s="140" t="inlineStr">
         <is>
           <t>NpvDemo</t>
         </is>
       </c>
-    </row>
-    <row r="25">
+      <c r="F24" s="133" t="inlineStr">
+        <is>
+          <t>Tahsilat Gecikme Toleransı</t>
+        </is>
+      </c>
+      <c r="G24" s="90" t="n"/>
+      <c r="H24" s="90" t="n"/>
+      <c r="I24" s="134" t="inlineStr">
+        <is>
+          <t>48 Gün Güvenli Eşik</t>
+        </is>
+      </c>
+      <c r="K24" s="141" t="inlineStr">
+        <is>
+          <t>Atıl kalan nakit rezervinin gecelik repoda</t>
+        </is>
+      </c>
+      <c r="L24" s="136" t="n"/>
+      <c r="M24" s="137" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
       <c r="A25" s="51" t="inlineStr">
         <is>
           <t>Gelir</t>
         </is>
       </c>
-      <c r="B25" s="52" t="n">
+      <c r="B25" s="142" t="n">
         <v>2898000</v>
       </c>
-      <c r="D25" s="51" t="inlineStr">
+      <c r="C25" s="90" t="n"/>
+      <c r="D25" s="139" t="inlineStr">
         <is>
           <t>İyimser</t>
         </is>
       </c>
-      <c r="E25" s="52" t="n">
+      <c r="E25" s="143" t="n">
         <v>3200000</v>
       </c>
-    </row>
-    <row r="26">
+      <c r="F25" s="113" t="inlineStr">
+        <is>
+          <t>██████████████████████████████ Güvenli Bölge (%100)</t>
+        </is>
+      </c>
+      <c r="G25" s="144" t="n"/>
+      <c r="H25" s="144" t="n"/>
+      <c r="I25" s="144" t="n"/>
+      <c r="K25" s="141" t="inlineStr">
+        <is>
+          <t>değerlendirilmesiyle ek getiri imkanı.</t>
+        </is>
+      </c>
+      <c r="L25" s="136" t="n"/>
+      <c r="M25" s="137" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="51" t="inlineStr">
         <is>
           <t>CAPEX</t>
         </is>
       </c>
-      <c r="B26" s="52" t="n">
+      <c r="B26" s="145" t="n">
         <v>4200000</v>
       </c>
-      <c r="D26" s="51" t="inlineStr">
+      <c r="C26" s="90" t="n"/>
+      <c r="D26" s="139" t="inlineStr">
         <is>
           <t>Baz</t>
         </is>
       </c>
-      <c r="E26" s="52" t="n">
+      <c r="E26" s="143" t="n">
         <v>1850000</v>
       </c>
-    </row>
-    <row r="27">
+      <c r="F26" s="146" t="inlineStr">
+        <is>
+          <t>✓ 90 GÜNLÜK PROJEKSİYONDA NAKİT SIKIŞIKLIĞI TESPİT EDİLMEDİ</t>
+        </is>
+      </c>
+      <c r="G26" s="147" t="n"/>
+      <c r="H26" s="147" t="n"/>
+      <c r="I26" s="147" t="n"/>
+      <c r="K26" s="148" t="inlineStr">
+        <is>
+          <t>FONLAMA SENARYOSUNU İNCELE ›</t>
+        </is>
+      </c>
+      <c r="L26" s="114" t="n"/>
+      <c r="M26" s="114" t="n"/>
+    </row>
+    <row r="27" ht="26" customHeight="1">
       <c r="A27" s="51" t="inlineStr">
         <is>
           <t>NPV</t>
         </is>
       </c>
-      <c r="B27" s="52" t="n">
+      <c r="B27" s="149" t="n">
         <v>1850000</v>
       </c>
-      <c r="D27" s="51" t="inlineStr">
+      <c r="C27" s="99" t="n"/>
+      <c r="D27" s="150" t="inlineStr">
         <is>
           <t>Kötümser</t>
         </is>
       </c>
-      <c r="E27" s="52" t="n">
+      <c r="E27" s="151" t="n">
         <v>-420000</v>
       </c>
-    </row>
-    <row r="28"/>
+      <c r="F27" s="152" t="n"/>
+      <c r="G27" s="99" t="n"/>
+      <c r="H27" s="99" t="n"/>
+      <c r="I27" s="100" t="n"/>
+      <c r="K27" s="153" t="n"/>
+      <c r="L27" s="154" t="n"/>
+      <c r="M27" s="155" t="n"/>
+    </row>
     <row r="29">
       <c r="A29" s="51" t="inlineStr">
         <is>
@@ -23439,16 +24245,16 @@
   <mergeCells count="13">
     <mergeCell ref="D14:J14"/>
     <mergeCell ref="B22:H22"/>
-    <mergeCell ref="D11:J11"/>
     <mergeCell ref="D18:J18"/>
     <mergeCell ref="D17:J17"/>
-    <mergeCell ref="D12:J12"/>
     <mergeCell ref="D20:J20"/>
     <mergeCell ref="D16:J16"/>
     <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B2:K2"/>
     <mergeCell ref="D15:J15"/>
     <mergeCell ref="D19:J19"/>
     <mergeCell ref="D13:J13"/>
+    <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">

</xml_diff>